<commit_message>
feat(dashboard): extend date range to 30 days and add fix_dates
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15.01.2024</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">

</xml_diff>